<commit_message>
Fix LS and FSS logic in PAL signal analysis table
LS was incorrectly A for lines 1-2 and 6-8 (pre-eq and post-eq).
Fixed: LS=NA for all of v_cnt 0-7 (lines 1-8); all special pulse
regions (pre-eq, broad, post-eq) replace the standard H-sync.

FSS was incorrectly Half Signal for line 8 (v_cnt=7).
Fixed: FSS=A for full lines 4-8 per VHDL plain range check.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017hYU7zmWoUoe7kPyUjvHZ6
</commit_message>
<xml_diff>
--- a/docs/PAL_Signal_Analysis.xlsx
+++ b/docs/PAL_Signal_Analysis.xlsx
@@ -39,13 +39,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00999999"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00999999"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -151,37 +151,37 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -652,40 +652,40 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -697,40 +697,40 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -740,42 +740,42 @@
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Half Signal</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Half Signal</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>Half Signal</t>
         </is>
@@ -785,42 +785,42 @@
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -830,42 +830,42 @@
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -875,9 +875,9 @@
       <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -890,7 +890,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -905,12 +905,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -920,9 +920,9 @@
       <c r="A8" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -935,7 +935,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -950,12 +950,12 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -965,42 +965,42 @@
       <c r="A9" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Half Signal</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Half Signal</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1015,7 +1015,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1025,7 +1025,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1035,17 +1035,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1060,7 +1060,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1070,7 +1070,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1080,17 +1080,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1105,7 +1105,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1115,7 +1115,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1125,17 +1125,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1150,7 +1150,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1160,7 +1160,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1170,17 +1170,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1195,7 +1195,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1205,7 +1205,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1215,17 +1215,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1240,7 +1240,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1250,7 +1250,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1260,17 +1260,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1285,7 +1285,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1295,7 +1295,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1305,17 +1305,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1330,7 +1330,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1340,7 +1340,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1350,17 +1350,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1375,7 +1375,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1385,7 +1385,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1395,17 +1395,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1420,7 +1420,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1430,7 +1430,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1440,17 +1440,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1465,7 +1465,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1475,7 +1475,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1485,17 +1485,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1510,7 +1510,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1520,7 +1520,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1530,17 +1530,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1555,7 +1555,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1565,7 +1565,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1575,17 +1575,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1600,7 +1600,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1610,7 +1610,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1620,17 +1620,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1645,7 +1645,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1655,7 +1655,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1665,17 +1665,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1690,7 +1690,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1700,7 +1700,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1710,17 +1710,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1735,7 +1735,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1745,7 +1745,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1755,17 +1755,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1780,7 +1780,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1795,22 +1795,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1825,7 +1825,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1840,22 +1840,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1870,7 +1870,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1885,22 +1885,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1915,7 +1915,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1930,22 +1930,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1960,7 +1960,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1975,22 +1975,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2005,7 +2005,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2020,22 +2020,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2050,7 +2050,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2060,7 +2060,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2070,17 +2070,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2095,7 +2095,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2105,7 +2105,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2115,17 +2115,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2140,7 +2140,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2150,7 +2150,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2160,17 +2160,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2185,7 +2185,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2200,22 +2200,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2230,7 +2230,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2245,22 +2245,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2275,7 +2275,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2290,22 +2290,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2320,7 +2320,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2335,22 +2335,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2365,7 +2365,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2380,22 +2380,22 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2410,7 +2410,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2420,7 +2420,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2430,17 +2430,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Redesign PAL signal table: 4-state per-half-line format
Replace A/NA/Half Signal with Full / 1st Half / 2nd Half / NA so each
cell shows WHERE on the line the signal is active, not just whether.

Key corrections:
- LS = 1st Half on normal lines (H-sync at h_cnt 16..62, always 1st half)
- Pre/Broad/Post show 1st Half or 2nd Half for mixed lines (scope line 3 and 8)
- CB = 1st Half for active video lines (H-blank h_cnt 0..119 only)
- Video = Full for active lines (h_cnt 120..639 spans both halves)
- Fix H_ACT_S constant to 120 (was 144; VHDL = H_FRONT+H_SYNC_W+H_BACK = 16+47+57)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017hYU7zmWoUoe7kPyUjvHZ6
</commit_message>
<xml_diff>
--- a/docs/PAL_Signal_Analysis.xlsx
+++ b/docs/PAL_Signal_Analysis.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAL F1 Signal States" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAL Signal States" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,20 +51,27 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="007F4F00"/>
+      <color rgb="007F3300"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005C3D00"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +96,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCC80"/>
       </patternFill>
     </fill>
     <fill>
@@ -143,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -166,60 +178,87 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -588,18 +627,18 @@
   <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Line</t>
@@ -646,7 +685,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="17" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -662,7 +701,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -672,7 +711,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -687,11 +726,11 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -707,7 +746,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -717,7 +756,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -732,11 +771,11 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
+          <t>Full</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
@@ -752,7 +791,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -762,7 +801,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -772,16 +811,16 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Half Signal</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
-        <is>
-          <t>Half Signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
+          <t>2nd Half</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
@@ -792,12 +831,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -807,7 +846,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -817,7 +856,7 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -826,7 +865,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1">
+    <row r="6" ht="17" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
@@ -837,12 +876,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -852,7 +891,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -862,7 +901,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -871,8 +910,8 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="8" t="n">
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -880,14 +919,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -895,14 +934,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -916,8 +955,8 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="8" t="n">
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="9" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -925,14 +964,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -940,14 +979,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -961,8 +1000,8 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="8" t="n">
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -970,14 +1009,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -985,14 +1024,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Half Signal</t>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1006,13 +1045,13 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="10" t="n">
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1020,9 +1059,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1030,9 +1069,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1051,13 +1090,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="10" t="n">
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1065,9 +1104,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1075,9 +1114,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1096,13 +1135,13 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="10" t="n">
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1110,9 +1149,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1120,9 +1159,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1141,13 +1180,13 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="10" t="n">
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1155,9 +1194,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1165,9 +1204,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1186,13 +1225,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="10" t="n">
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1200,9 +1239,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1210,9 +1249,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1231,13 +1270,13 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="10" t="n">
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1245,9 +1284,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1255,9 +1294,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1276,13 +1315,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="10" t="n">
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1290,9 +1329,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1300,9 +1339,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1321,13 +1360,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="10" t="n">
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1335,9 +1374,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1345,9 +1384,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1366,13 +1405,13 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="10" t="n">
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1380,9 +1419,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1390,9 +1429,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1411,13 +1450,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="10" t="n">
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1425,9 +1464,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1435,9 +1474,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1456,13 +1495,13 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="10" t="n">
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1470,9 +1509,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1480,9 +1519,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1501,13 +1540,13 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="10" t="n">
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1515,9 +1554,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1525,9 +1564,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1546,13 +1585,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="10" t="n">
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1560,9 +1599,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1570,9 +1609,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1591,13 +1630,13 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="10" t="n">
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1605,9 +1644,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1615,9 +1654,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1636,13 +1675,13 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="10" t="n">
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1650,9 +1689,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1660,9 +1699,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1681,13 +1720,13 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="10" t="n">
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1695,9 +1734,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1705,9 +1744,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1726,13 +1765,13 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="10" t="n">
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1740,9 +1779,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1750,9 +1789,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1771,13 +1810,13 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="12" t="n">
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="13" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1785,14 +1824,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1816,13 +1855,13 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="12" t="n">
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="13" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1830,14 +1869,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1861,13 +1900,13 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="12" t="n">
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="13" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1875,14 +1914,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1906,13 +1945,13 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="12" t="n">
-        <v>310</v>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="13" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1920,14 +1959,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1951,13 +1990,13 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="12" t="n">
+    <row r="31" ht="17" customHeight="1">
+      <c r="A31" s="13" t="n">
         <v>311</v>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1965,14 +2004,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1996,13 +2035,13 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="12" t="n">
+    <row r="32" ht="17" customHeight="1">
+      <c r="A32" s="13" t="n">
         <v>312</v>
       </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2010,14 +2049,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D32" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E32" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2041,13 +2080,13 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="10" t="n">
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" s="11" t="n">
         <v>313</v>
       </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2055,9 +2094,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -2065,9 +2104,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2086,13 +2125,13 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="10" t="n">
-        <v>336</v>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+    <row r="34" ht="17" customHeight="1">
+      <c r="A34" s="11" t="n">
+        <v>314</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2100,9 +2139,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2110,9 +2149,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F34" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -2131,13 +2170,13 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="10" t="n">
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="11" t="n">
         <v>337</v>
       </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2145,9 +2184,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2155,9 +2194,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2176,13 +2215,13 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="12" t="n">
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="13" t="n">
         <v>338</v>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2190,14 +2229,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E36" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2221,13 +2260,13 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="12" t="n">
+    <row r="37" ht="17" customHeight="1">
+      <c r="A37" s="13" t="n">
         <v>339</v>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2235,14 +2274,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2266,13 +2305,13 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="12" t="n">
-        <v>622</v>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+    <row r="38" ht="17" customHeight="1">
+      <c r="A38" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2280,14 +2319,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -2311,13 +2350,13 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="12" t="n">
+    <row r="39" ht="17" customHeight="1">
+      <c r="A39" s="13" t="n">
         <v>623</v>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2325,14 +2364,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E39" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -2356,13 +2395,13 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="12" t="n">
+    <row r="40" ht="17" customHeight="1">
+      <c r="A40" s="13" t="n">
         <v>624</v>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2370,14 +2409,14 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E40" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2401,13 +2440,13 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="10" t="n">
+    <row r="41" ht="17" customHeight="1">
+      <c r="A41" s="11" t="n">
         <v>625</v>
       </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2415,9 +2454,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D41" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -2425,9 +2464,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F41" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -2457,118 +2496,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B1" s="15" t="inlineStr">
-        <is>
-          <t>Applicable — signal is fully active this line</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>Not applicable — signal is inactive</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="18" t="inlineStr">
-        <is>
-          <t>Half Signal</t>
-        </is>
-      </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>Active for approx half the line (sub-line event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="20" t="inlineStr"/>
-      <c r="B4" s="21" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>Row colours</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+    <row r="1" ht="17" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="17" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Signal active for entire line (both halves)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Signal active in 1st half only  (h_cnt 0..319)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>2nd Half</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Signal active in 2nd half only  (h_cnt 320..639)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Signal not active on this line</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="25" t="inlineStr"/>
+      <c r="B6" s="26" t="inlineStr"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Row colour</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Pink</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>Pre-equalising pulses (v_cnt 0-2 first half)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Pre-equalising region  (v_cnt 0-1, first half of 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Orange</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
-        <is>
-          <t>Broad sync pulses (v_cnt 2 second half – 4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Broad sync region      (v_cnt 2 2nd half, 3, 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Lavender</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>Post-equalising pulses (v_cnt 5-7 first half)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Post-equalising region (v_cnt 5-6, first half of 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>Light grey</t>
         </is>
       </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>Blanked non-sync lines (VBI lines 8-24)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>VBI blank lines        (v_cnt 8 .. V_ACT_S_F1-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Light green</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Active video lines (F1 25-311, F2 337-623)</t>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Active video lines     (F1 v25-311, F2 v337-623)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add F2 sync region (Pre/Broad/Post) to PAL signal table
F2 VBI sync is offset by half a line vs F1 (interlaced).
Adds scope lines 313-321 covering the full F2 sync sequence:
  v_cnt=312 (line 313): LS=1st Half, Pre=2nd Half  (mixed: H-sync then pre-eq)
  v_cnt=313,314        : Pre=Full
  v_cnt=315,316        : Broad=Full, FSS F2 starts (2nd Half on line 316)
  v_cnt=317            : Broad=1st Half, Post=2nd Half  (mixed)
  v_cnt=318,319        : Post=Full
  v_cnt=320 (line 321) : LS=1st Half, FSS=1st Half  (FSS ends mid-line)

Also adds FSS F2 constants and row colours for F2 sync region.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017hYU7zmWoUoe7kPyUjvHZ6
</commit_message>
<xml_diff>
--- a/docs/PAL_Signal_Analysis.xlsx
+++ b/docs/PAL_Signal_Analysis.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2081,7 +2081,7 @@
       </c>
     </row>
     <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="11" t="n">
+      <c r="A33" s="5" t="n">
         <v>313</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -2094,7 +2094,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
@@ -2104,7 +2104,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
@@ -2119,19 +2119,19 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>2nd Half</t>
         </is>
       </c>
     </row>
     <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="11" t="n">
+      <c r="A34" s="2" t="n">
         <v>314</v>
       </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2139,7 +2139,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
@@ -2149,7 +2149,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
@@ -2164,19 +2164,19 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
     </row>
     <row r="35" ht="17" customHeight="1">
-      <c r="A35" s="11" t="n">
-        <v>337</v>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
+      <c r="A35" s="2" t="n">
+        <v>315</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2184,7 +2184,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
@@ -2194,7 +2194,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F35" s="12" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Full</t>
         </is>
@@ -2209,39 +2209,39 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
     </row>
     <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="13" t="n">
-        <v>338</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="E36" s="14" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="A36" s="5" t="n">
+        <v>316</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>2nd Half</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -2249,9 +2249,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2261,32 +2261,32 @@
       </c>
     </row>
     <row r="37" ht="17" customHeight="1">
-      <c r="A37" s="13" t="n">
-        <v>339</v>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="E37" s="14" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="A37" s="5" t="n">
+        <v>317</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2294,9 +2294,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2306,42 +2306,42 @@
       </c>
     </row>
     <row r="38" ht="17" customHeight="1">
-      <c r="A38" s="13" t="n">
-        <v>340</v>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="A38" s="9" t="n">
+        <v>318</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>2nd Half</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2351,37 +2351,37 @@
       </c>
     </row>
     <row r="39" ht="17" customHeight="1">
-      <c r="A39" s="13" t="n">
-        <v>623</v>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="E39" s="14" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="A39" s="9" t="n">
+        <v>319</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2396,37 +2396,37 @@
       </c>
     </row>
     <row r="40" ht="17" customHeight="1">
-      <c r="A40" s="13" t="n">
-        <v>624</v>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="E40" s="14" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="A40" s="9" t="n">
+        <v>320</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>Full</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2442,44 +2442,359 @@
     </row>
     <row r="41" ht="17" customHeight="1">
       <c r="A41" s="11" t="n">
+        <v>321</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="11" t="n">
+        <v>337</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="17" customHeight="1">
+      <c r="A43" s="13" t="n">
+        <v>338</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="17" customHeight="1">
+      <c r="A44" s="13" t="n">
+        <v>339</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="17" customHeight="1">
+      <c r="A45" s="13" t="n">
+        <v>340</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="17" customHeight="1">
+      <c r="A46" s="13" t="n">
+        <v>623</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="17" customHeight="1">
+      <c r="A47" s="13" t="n">
+        <v>624</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="17" customHeight="1">
+      <c r="A48" s="11" t="n">
         <v>625</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>1st Half</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>1st Half</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>